<commit_message>
generator added, fix types.py  new tests
</commit_message>
<xml_diff>
--- a/data/tracking/mock_paper_planner.xlsx
+++ b/data/tracking/mock_paper_planner.xlsx
@@ -2848,7 +2848,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>encrypt using given key stream; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling</t>
+          <t>encrypt using given key stream; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -2961,12 +2961,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>encrypt using key and tableau; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>encrypt using key and tableau; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -3020,12 +3020,12 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>decrypt using keyword and tableau; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>decrypt using keyword and tableau; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -3291,7 +3291,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>explain with example; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>explain with example; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -3344,7 +3344,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>explain with example; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>explain with example; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -3988,7 +3988,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>describe similarities and differences; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>describe similarities and differences; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -4041,7 +4041,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>describe steps; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>describe steps; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -4425,7 +4425,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>State final encoded result; recovered by cleaning pass; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>State final encoded result; recovered by cleaning pass; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -4586,7 +4586,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>explain relationship; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>explain relationship; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -4803,7 +4803,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>calculate U; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>calculate U; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -4861,7 +4861,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>find row index; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>find row index; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -5179,7 +5179,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>explain concept; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>explain concept; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -5285,7 +5285,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>definition; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>definition; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -5391,7 +5391,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>scenario-based explanation; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>scenario-based explanation; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -5511,7 +5511,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>calculate subkey; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling</t>
+          <t>calculate subkey; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -5569,7 +5569,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>calculate left half; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling</t>
+          <t>calculate left half; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -5627,7 +5627,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>calculate right half; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling</t>
+          <t>calculate right half; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -5682,7 +5682,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>calculate key; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling</t>
+          <t>calculate key; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -5740,7 +5740,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>calculate IP; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling</t>
+          <t>calculate IP; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -5798,7 +5798,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>calculate R0; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling</t>
+          <t>calculate R0; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -5856,7 +5856,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>calculate expansion; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling</t>
+          <t>calculate expansion; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -5911,7 +5911,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>calculate block; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling</t>
+          <t>calculate block; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -5969,7 +5969,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>find column index; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling</t>
+          <t>find column index; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -6027,7 +6027,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>find output value; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling</t>
+          <t>find output value; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling; topic inherited from sibling; compute task inherited from sibling</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -6260,7 +6260,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>explain with diagram; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>explain with diagram; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -6641,7 +6641,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>define term; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>define term; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -6694,7 +6694,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>propose solution for scenario; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>propose solution for scenario; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -6800,7 +6800,7 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>list examples; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>list examples; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
@@ -7130,7 +7130,7 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>explain concept; recovered by cleaning pass; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>explain concept; recovered by cleaning pass; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -7236,7 +7236,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>list examples; recovered by cleaning pass; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>list examples; recovered by cleaning pass; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -7515,7 +7515,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>calculate DES IP and L values; recovered by cleaning pass; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling</t>
+          <t>calculate DES IP and L values; recovered by cleaning pass; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -7677,7 +7677,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>explain examples; recovered by cleaning pass; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>explain examples; recovered by cleaning pass; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -7730,7 +7730,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>explain impact; recovered by cleaning pass; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>explain impact; recovered by cleaning pass; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -8111,7 +8111,7 @@
       </c>
       <c r="J104" t="inlineStr">
         <is>
-          <t>show methods step by step; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>show methods step by step; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K104" t="inlineStr">
@@ -8165,7 +8165,7 @@
       </c>
       <c r="J105" t="inlineStr">
         <is>
-          <t>determine and state reason; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>determine and state reason; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K105" t="inlineStr">
@@ -8282,7 +8282,7 @@
       </c>
       <c r="J107" t="inlineStr">
         <is>
-          <t>find row index i; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>find row index i; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K107" t="inlineStr">
@@ -8388,7 +8388,7 @@
       </c>
       <c r="J109" t="inlineStr">
         <is>
-          <t>explain in own words; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>explain in own words; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K109" t="inlineStr">
@@ -10964,7 +10964,7 @@
       </c>
       <c r="J156" t="inlineStr">
         <is>
-          <t>Opinion and explanation; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>Opinion and explanation; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K156" t="inlineStr">
@@ -11173,7 +11173,7 @@
       </c>
       <c r="J160" t="inlineStr">
         <is>
-          <t>Classify violation; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>Classify violation; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K160" t="inlineStr">
@@ -11279,7 +11279,7 @@
       </c>
       <c r="J162" t="inlineStr">
         <is>
-          <t>Classify violation; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>Classify violation; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K162" t="inlineStr">
@@ -11332,7 +11332,7 @@
       </c>
       <c r="J163" t="inlineStr">
         <is>
-          <t>Classify violation; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>Classify violation; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K163" t="inlineStr">
@@ -11385,7 +11385,7 @@
       </c>
       <c r="J164" t="inlineStr">
         <is>
-          <t>Classify violation; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>Classify violation; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K164" t="inlineStr">
@@ -11706,7 +11706,7 @@
       </c>
       <c r="J170" t="inlineStr">
         <is>
-          <t>Explain your answer; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>Explain your answer; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K170" t="inlineStr">
@@ -12452,7 +12452,7 @@
       </c>
       <c r="J184" t="inlineStr">
         <is>
-          <t>What do they have in common; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>What do they have in common; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K184" t="inlineStr">
@@ -12558,7 +12558,7 @@
       </c>
       <c r="J186" t="inlineStr">
         <is>
-          <t>Why is this principle important; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>Why is this principle important; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K186" t="inlineStr">
@@ -13250,7 +13250,7 @@
       </c>
       <c r="J199" t="inlineStr">
         <is>
-          <t>classify as mechanism or policy; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>classify as mechanism or policy; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K199" t="inlineStr">
@@ -13303,7 +13303,7 @@
       </c>
       <c r="J200" t="inlineStr">
         <is>
-          <t>classify as mechanism or policy; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>classify as mechanism or policy; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K200" t="inlineStr">
@@ -13567,7 +13567,7 @@
       </c>
       <c r="J205" t="inlineStr">
         <is>
-          <t>suggest and explain biometric method; low block coverage - check sub-parts are complete; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>suggest and explain biometric method; low block coverage - check sub-parts are complete; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K205" t="inlineStr">
@@ -13620,7 +13620,7 @@
       </c>
       <c r="J206" t="inlineStr">
         <is>
-          <t>suggest and explain biometric method; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>suggest and explain biometric method; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K206" t="inlineStr">
@@ -15250,7 +15250,7 @@
       </c>
       <c r="J237" t="inlineStr">
         <is>
-          <t>Illustrate using node and arrow; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>Illustrate using node and arrow; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K237" t="inlineStr">
@@ -15366,7 +15366,7 @@
       </c>
       <c r="J239" t="inlineStr">
         <is>
-          <t>Illustrate using node and arrow; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>Illustrate using node and arrow; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K239" t="inlineStr">
@@ -15638,7 +15638,7 @@
       </c>
       <c r="J244" t="inlineStr">
         <is>
-          <t>List one disadvantage; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>List one disadvantage; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K244" t="inlineStr">
@@ -16528,12 +16528,12 @@
       </c>
       <c r="I261" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="J261" t="inlineStr">
         <is>
-          <t>Encrypt using provided table; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>Encrypt using provided table; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K261" t="inlineStr">
@@ -17184,7 +17184,7 @@
       </c>
       <c r="J273" t="inlineStr">
         <is>
-          <t>write pseudo-code; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling</t>
+          <t>write pseudo-code; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling</t>
         </is>
       </c>
       <c r="K273" t="inlineStr">
@@ -17286,12 +17286,12 @@
       </c>
       <c r="I275" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="J275" t="inlineStr">
         <is>
-          <t>describe with example; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling</t>
+          <t>describe with example; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K275" t="inlineStr">
@@ -17705,7 +17705,7 @@
       </c>
       <c r="J283" t="inlineStr">
         <is>
-          <t>apply rules and explain; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>apply rules and explain; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K283" t="inlineStr">
@@ -17905,7 +17905,7 @@
       </c>
       <c r="J287" t="inlineStr">
         <is>
-          <t>define strategies; low block coverage - check sub-parts are complete; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>define strategies; low block coverage - check sub-parts are complete; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K287" t="inlineStr">
@@ -18011,7 +18011,7 @@
       </c>
       <c r="J289" t="inlineStr">
         <is>
-          <t>identify specific principles; low block coverage - check sub-parts are complete; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>identify specific principles; low block coverage - check sub-parts are complete; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K289" t="inlineStr">
@@ -18064,7 +18064,7 @@
       </c>
       <c r="J290" t="inlineStr">
         <is>
-          <t>discuss previously identified principles; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>discuss previously identified principles; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K290" t="inlineStr">
@@ -18576,7 +18576,7 @@
       </c>
       <c r="J300" t="inlineStr">
         <is>
-          <t>explain mechanism design; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>explain mechanism design; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K300" t="inlineStr">
@@ -18899,7 +18899,7 @@
       </c>
       <c r="J306" t="inlineStr">
         <is>
-          <t>discuss advantages; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>discuss advantages; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K306" t="inlineStr">
@@ -19525,7 +19525,7 @@
       </c>
       <c r="J318" t="inlineStr">
         <is>
-          <t>perform encryption calculation; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>perform encryption calculation; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K318" t="inlineStr">
@@ -19578,7 +19578,7 @@
       </c>
       <c r="J319" t="inlineStr">
         <is>
-          <t>perform decryption calculation; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>perform decryption calculation; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K319" t="inlineStr">
@@ -19679,7 +19679,7 @@
       </c>
       <c r="J321" t="inlineStr">
         <is>
-          <t>definition; low block coverage - check sub-parts are complete; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>definition; low block coverage - check sub-parts are complete; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K321" t="inlineStr">
@@ -19732,7 +19732,7 @@
       </c>
       <c r="J322" t="inlineStr">
         <is>
-          <t>explain with example; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>explain with example; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K322" t="inlineStr">
@@ -20103,7 +20103,7 @@
       </c>
       <c r="J329" t="inlineStr">
         <is>
-          <t>design strategy; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>design strategy; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K329" t="inlineStr">
@@ -20310,7 +20310,7 @@
       </c>
       <c r="J333" t="inlineStr">
         <is>
-          <t>discuss combination; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>discuss combination; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K333" t="inlineStr">
@@ -20628,7 +20628,7 @@
       </c>
       <c r="J339" t="inlineStr">
         <is>
-          <t>differentiate substitution and transposition; low block coverage - check sub-parts are complete; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>differentiate substitution and transposition; low block coverage - check sub-parts are complete; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K339" t="inlineStr">
@@ -20782,7 +20782,7 @@
       </c>
       <c r="J342" t="inlineStr">
         <is>
-          <t>Classify as violation of confidentiality, integrity, availability or combination; marks computed by code from '(N marks)' after quote; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>Classify as violation of confidentiality, integrity, availability or combination; marks computed by code from '(N marks)' after quote; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K342" t="inlineStr">
@@ -20888,7 +20888,7 @@
       </c>
       <c r="J344" t="inlineStr">
         <is>
-          <t>Classify as violation of confidentiality, integrity, availability or combination; marks computed by code from '(N marks)' after quote; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>Classify as violation of confidentiality, integrity, availability or combination; marks computed by code from '(N marks)' after quote; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K344" t="inlineStr">
@@ -20941,7 +20941,7 @@
       </c>
       <c r="J345" t="inlineStr">
         <is>
-          <t>Classify as violation of confidentiality, integrity, availability or combination; marks computed by code from '(N marks)' after quote; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>Classify as violation of confidentiality, integrity, availability or combination; marks computed by code from '(N marks)' after quote; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K345" t="inlineStr">
@@ -20994,7 +20994,7 @@
       </c>
       <c r="J346" t="inlineStr">
         <is>
-          <t>Classify as violation of confidentiality, integrity, availability or combination; marks computed by code from '(N marks)' after quote; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>Classify as violation of confidentiality, integrity, availability or combination; marks computed by code from '(N marks)' after quote; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K346" t="inlineStr">
@@ -21153,7 +21153,7 @@
       </c>
       <c r="J349" t="inlineStr">
         <is>
-          <t>Write pseudo-code; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling</t>
+          <t>Write pseudo-code; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling</t>
         </is>
       </c>
       <c r="K349" t="inlineStr">
@@ -21406,7 +21406,7 @@
       </c>
       <c r="J354" t="inlineStr">
         <is>
-          <t>Discuss TWO advantages; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>Discuss TWO advantages; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K354" t="inlineStr">
@@ -21512,7 +21512,7 @@
       </c>
       <c r="J356" t="inlineStr">
         <is>
-          <t>Identify the importance; quote fuzzy-matched to paper; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>Identify the importance; quote fuzzy-matched to paper; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K356" t="inlineStr">
@@ -22533,7 +22533,7 @@
       </c>
       <c r="J376" t="inlineStr">
         <is>
-          <t>decrypt to verify; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling</t>
+          <t>decrypt to verify; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K376" t="inlineStr">
@@ -23282,7 +23282,7 @@
       </c>
       <c r="J391" t="inlineStr">
         <is>
-          <t>draw diagram; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>draw diagram; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K391" t="inlineStr">
@@ -23383,12 +23383,12 @@
       </c>
       <c r="I393" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="J393" t="inlineStr">
         <is>
-          <t>encrypt message show work; inputs inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling</t>
+          <t>encrypt message show work; inputs inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K393" t="inlineStr">
@@ -23653,7 +23653,7 @@
       </c>
       <c r="J398" t="inlineStr">
         <is>
-          <t>suggest biometric method; low block coverage - check sub-parts are complete; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>suggest biometric method; low block coverage - check sub-parts are complete; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K398" t="inlineStr">
@@ -23860,7 +23860,7 @@
       </c>
       <c r="J402" t="inlineStr">
         <is>
-          <t>explain weaknesses; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>explain weaknesses; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K402" t="inlineStr">
@@ -24572,7 +24572,7 @@
       </c>
       <c r="J416" t="inlineStr">
         <is>
-          <t>classify violation type; marks computed by code from '(N marks)' after quote; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>classify violation type; marks computed by code from '(N marks)' after quote; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K416" t="inlineStr">
@@ -24625,7 +24625,7 @@
       </c>
       <c r="J417" t="inlineStr">
         <is>
-          <t>classify violation type; marks computed by code from '(N marks)' after quote; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>classify violation type; marks computed by code from '(N marks)' after quote; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K417" t="inlineStr">
@@ -24678,7 +24678,7 @@
       </c>
       <c r="J418" t="inlineStr">
         <is>
-          <t>classify violation type; marks computed by code from '(N marks)' after quote; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>classify violation type; marks computed by code from '(N marks)' after quote; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K418" t="inlineStr">
@@ -24731,7 +24731,7 @@
       </c>
       <c r="J419" t="inlineStr">
         <is>
-          <t>classify violation type; marks computed by code from '(N marks)' after quote; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>classify violation type; marks computed by code from '(N marks)' after quote; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K419" t="inlineStr">
@@ -24784,7 +24784,7 @@
       </c>
       <c r="J420" t="inlineStr">
         <is>
-          <t>classify violation type; marks computed by code from '(N marks)' after quote; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>classify violation type; marks computed by code from '(N marks)' after quote; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K420" t="inlineStr">
@@ -24996,7 +24996,7 @@
       </c>
       <c r="J424" t="inlineStr">
         <is>
-          <t>explain based on scenario; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>explain based on scenario; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K424" t="inlineStr">
@@ -25314,7 +25314,7 @@
       </c>
       <c r="J430" t="inlineStr">
         <is>
-          <t>write pseudo-code; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling</t>
+          <t>write pseudo-code; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling</t>
         </is>
       </c>
       <c r="K430" t="inlineStr">
@@ -25362,12 +25362,12 @@
       </c>
       <c r="I431" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="J431" t="inlineStr">
         <is>
-          <t>encrypt and show work; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>encrypt and show work; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K431" t="inlineStr">
@@ -26229,7 +26229,7 @@
       </c>
       <c r="J448" t="inlineStr">
         <is>
-          <t>classify violation type; quote fuzzy-matched to paper; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>classify violation type; quote fuzzy-matched to paper; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K448" t="inlineStr">
@@ -26282,7 +26282,7 @@
       </c>
       <c r="J449" t="inlineStr">
         <is>
-          <t>classify violation type; marks computed by code from '(N marks)' after quote; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>classify violation type; marks computed by code from '(N marks)' after quote; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K449" t="inlineStr">
@@ -26335,7 +26335,7 @@
       </c>
       <c r="J450" t="inlineStr">
         <is>
-          <t>classify violation type; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>classify violation type; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K450" t="inlineStr">
@@ -26547,7 +26547,7 @@
       </c>
       <c r="J454" t="inlineStr">
         <is>
-          <t>explain principles; low block coverage - check sub-parts are complete; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>explain principles; low block coverage - check sub-parts are complete; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K454" t="inlineStr">
@@ -26797,7 +26797,7 @@
       </c>
       <c r="J459" t="inlineStr">
         <is>
-          <t>extract fields from string; quote fuzzy-matched to paper; recovered by cleaning pass; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>extract fields from string; quote fuzzy-matched to paper; recovered by cleaning pass; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K459" t="inlineStr">
@@ -27527,7 +27527,7 @@
       </c>
       <c r="J473" t="inlineStr">
         <is>
-          <t>Define terminology; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>Define terminology; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K473" t="inlineStr">
@@ -27577,7 +27577,7 @@
       </c>
       <c r="J474" t="inlineStr">
         <is>
-          <t>Define terminology; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>Define terminology; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K474" t="inlineStr">
@@ -27842,7 +27842,7 @@
       </c>
       <c r="J479" t="inlineStr">
         <is>
-          <t>Explain based on scenario; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>Explain based on scenario; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K479" t="inlineStr">
@@ -28142,7 +28142,7 @@
       </c>
       <c r="J485" t="inlineStr">
         <is>
-          <t>Give examples; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>Give examples; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K485" t="inlineStr">
@@ -28659,7 +28659,7 @@
       </c>
       <c r="J495" t="inlineStr">
         <is>
-          <t>Define and give example; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>Define and give example; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K495" t="inlineStr">
@@ -29035,7 +29035,7 @@
       </c>
       <c r="J502" t="inlineStr">
         <is>
-          <t>define meaning; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>define meaning; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K502" t="inlineStr">
@@ -29189,7 +29189,7 @@
       </c>
       <c r="J505" t="inlineStr">
         <is>
-          <t>identify actions; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>identify actions; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K505" t="inlineStr">
@@ -29295,7 +29295,7 @@
       </c>
       <c r="J507" t="inlineStr">
         <is>
-          <t>explain difference; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>explain difference; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K507" t="inlineStr">
@@ -29401,7 +29401,7 @@
       </c>
       <c r="J509" t="inlineStr">
         <is>
-          <t>state and suggest; marks computed by code from '(N marks)' after quote; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>state and suggest; marks computed by code from '(N marks)' after quote; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K509" t="inlineStr">
@@ -29454,7 +29454,7 @@
       </c>
       <c r="J510" t="inlineStr">
         <is>
-          <t>state and suggest; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>state and suggest; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K510" t="inlineStr">
@@ -29976,7 +29976,7 @@
       </c>
       <c r="J520" t="inlineStr">
         <is>
-          <t>draw diagram; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>draw diagram; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K520" t="inlineStr">
@@ -30034,7 +30034,7 @@
       </c>
       <c r="J521" t="inlineStr">
         <is>
-          <t>draw diagram; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>draw diagram; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K521" t="inlineStr">
@@ -30188,7 +30188,7 @@
       </c>
       <c r="J524" t="inlineStr">
         <is>
-          <t>suggest and justify; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>suggest and justify; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K524" t="inlineStr">
@@ -30294,7 +30294,7 @@
       </c>
       <c r="J526" t="inlineStr">
         <is>
-          <t>identify components; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>identify components; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K526" t="inlineStr">
@@ -30442,7 +30442,7 @@
       </c>
       <c r="J529" t="inlineStr">
         <is>
-          <t>describe; low block coverage - check sub-parts are complete; recovered by cleaning pass; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>describe; low block coverage - check sub-parts are complete; recovered by cleaning pass; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K529" t="inlineStr">
@@ -30861,7 +30861,7 @@
       </c>
       <c r="J537" t="inlineStr">
         <is>
-          <t>list examples; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>list examples; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K537" t="inlineStr">
@@ -31329,7 +31329,7 @@
       </c>
       <c r="J546" t="inlineStr">
         <is>
-          <t>differentiate; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>differentiate; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K546" t="inlineStr">
@@ -31435,7 +31435,7 @@
       </c>
       <c r="J548" t="inlineStr">
         <is>
-          <t>briefly explain; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling</t>
+          <t>briefly explain; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling; inputs inherited from sibling</t>
         </is>
       </c>
       <c r="K548" t="inlineStr">
@@ -31536,12 +31536,12 @@
       </c>
       <c r="I550" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>Y</t>
         </is>
       </c>
       <c r="J550" t="inlineStr">
         <is>
-          <t>encrypt text; inputs inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling</t>
+          <t>encrypt text; inputs inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling; inputs inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K550" t="inlineStr">
@@ -31647,7 +31647,7 @@
       </c>
       <c r="J552" t="inlineStr">
         <is>
-          <t>define with example; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>define with example; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K552" t="inlineStr">
@@ -31859,7 +31859,7 @@
       </c>
       <c r="J556" t="inlineStr">
         <is>
-          <t>explain aspects; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>explain aspects; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K556" t="inlineStr">
@@ -32490,7 +32490,7 @@
       </c>
       <c r="J568" t="inlineStr">
         <is>
-          <t>definition question; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>definition question; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K568" t="inlineStr">
@@ -32702,7 +32702,7 @@
       </c>
       <c r="J572" t="inlineStr">
         <is>
-          <t>definition question; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>definition question; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K572" t="inlineStr">
@@ -32755,7 +32755,7 @@
       </c>
       <c r="J573" t="inlineStr">
         <is>
-          <t>reasoning question; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>reasoning question; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K573" t="inlineStr">
@@ -32813,7 +32813,7 @@
       </c>
       <c r="J574" t="inlineStr">
         <is>
-          <t>draw and explain; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>draw and explain; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K574" t="inlineStr">
@@ -33125,7 +33125,7 @@
       </c>
       <c r="J580" t="inlineStr">
         <is>
-          <t>identify similarities; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>identify similarities; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K580" t="inlineStr">
@@ -33493,7 +33493,7 @@
       </c>
       <c r="J587" t="inlineStr">
         <is>
-          <t>define term; marks computed by code from '(N marks)' after quote; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>define term; marks computed by code from '(N marks)' after quote; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K587" t="inlineStr">
@@ -33599,7 +33599,7 @@
       </c>
       <c r="J589" t="inlineStr">
         <is>
-          <t>define term; marks computed by code from '(N marks)' after quote; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>define term; marks computed by code from '(N marks)' after quote; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K589" t="inlineStr">
@@ -33652,7 +33652,7 @@
       </c>
       <c r="J590" t="inlineStr">
         <is>
-          <t>analyze scenario; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>analyze scenario; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K590" t="inlineStr">
@@ -33705,7 +33705,7 @@
       </c>
       <c r="J591" t="inlineStr">
         <is>
-          <t>comparison question; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>comparison question; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K591" t="inlineStr">
@@ -33758,7 +33758,7 @@
       </c>
       <c r="J592" t="inlineStr">
         <is>
-          <t>comparison question; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>comparison question; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K592" t="inlineStr">
@@ -34215,7 +34215,7 @@
       </c>
       <c r="J601" t="inlineStr">
         <is>
-          <t>opinion/suggestion; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>opinion/suggestion; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K601" t="inlineStr">
@@ -34427,7 +34427,7 @@
       </c>
       <c r="J605" t="inlineStr">
         <is>
-          <t>Definition question; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>Definition question; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K605" t="inlineStr">
@@ -34909,7 +34909,7 @@
       </c>
       <c r="J614" t="inlineStr">
         <is>
-          <t>Apply model rules to scenario; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>Apply model rules to scenario; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K614" t="inlineStr">
@@ -35953,7 +35953,7 @@
       </c>
       <c r="J634" t="inlineStr">
         <is>
-          <t>application/example based; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>application/example based; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K634" t="inlineStr">
@@ -36006,7 +36006,7 @@
       </c>
       <c r="J635" t="inlineStr">
         <is>
-          <t>discuss benefits; low block coverage - check sub-parts are complete; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>discuss benefits; low block coverage - check sub-parts are complete; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K635" t="inlineStr">
@@ -36847,7 +36847,7 @@
       </c>
       <c r="J651" t="inlineStr">
         <is>
-          <t>rank order; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>rank order; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K651" t="inlineStr">
@@ -37440,7 +37440,7 @@
       </c>
       <c r="J662" t="inlineStr">
         <is>
-          <t>justification required; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>justification required; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K662" t="inlineStr">
@@ -37705,7 +37705,7 @@
       </c>
       <c r="J667" t="inlineStr">
         <is>
-          <t>definition question; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>definition question; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K667" t="inlineStr">
@@ -37917,7 +37917,7 @@
       </c>
       <c r="J671" t="inlineStr">
         <is>
-          <t>definition question; low block coverage - check sub-parts are complete; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>definition question; low block coverage - check sub-parts are complete; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K671" t="inlineStr">
@@ -38771,7 +38771,7 @@
       </c>
       <c r="J687" t="inlineStr">
         <is>
-          <t>identify components from scenario; low block coverage - check sub-parts are complete; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>identify components from scenario; low block coverage - check sub-parts are complete; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K687" t="inlineStr">
@@ -39263,7 +39263,7 @@
       </c>
       <c r="J696" t="inlineStr">
         <is>
-          <t>explain with diagram; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>explain with diagram; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K696" t="inlineStr">
@@ -41422,7 +41422,7 @@
       </c>
       <c r="J736" t="inlineStr">
         <is>
-          <t>determine ethical element and justify; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>determine ethical element and justify; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K736" t="inlineStr">
@@ -43120,7 +43120,7 @@
       </c>
       <c r="J768" t="inlineStr">
         <is>
-          <t>describe three examples; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>describe three examples; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K768" t="inlineStr">
@@ -44550,7 +44550,7 @@
       </c>
       <c r="J795" t="inlineStr">
         <is>
-          <t>list all; low block coverage - check sub-parts are complete; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>list all; low block coverage - check sub-parts are complete; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K795" t="inlineStr">
@@ -44714,7 +44714,7 @@
       </c>
       <c r="J798" t="inlineStr">
         <is>
-          <t>determine ethical element and justify; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>determine ethical element and justify; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K798" t="inlineStr">
@@ -44979,7 +44979,7 @@
       </c>
       <c r="J803" t="inlineStr">
         <is>
-          <t>definition question; low block coverage - check sub-parts are complete; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>definition question; low block coverage - check sub-parts are complete; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K803" t="inlineStr">
@@ -46092,7 +46092,7 @@
       </c>
       <c r="J824" t="inlineStr">
         <is>
-          <t>explain mechanism; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>explain mechanism; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K824" t="inlineStr">
@@ -46940,7 +46940,7 @@
       </c>
       <c r="J840" t="inlineStr">
         <is>
-          <t>discuss components; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>discuss components; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K840" t="inlineStr">
@@ -47099,7 +47099,7 @@
       </c>
       <c r="J843" t="inlineStr">
         <is>
-          <t>state at least two; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>state at least two; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K843" t="inlineStr">
@@ -48249,7 +48249,7 @@
       </c>
       <c r="J865" t="inlineStr">
         <is>
-          <t>propose, explain mechanism and limitation; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>propose, explain mechanism and limitation; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K865" t="inlineStr">
@@ -48723,7 +48723,7 @@
       </c>
       <c r="J874" t="inlineStr">
         <is>
-          <t>compare, suggest and justify; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>compare, suggest and justify; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K874" t="inlineStr">
@@ -48935,7 +48935,7 @@
       </c>
       <c r="J878" t="inlineStr">
         <is>
-          <t>critically discuss and propose; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>critically discuss and propose; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K878" t="inlineStr">
@@ -48988,7 +48988,7 @@
       </c>
       <c r="J879" t="inlineStr">
         <is>
-          <t>explain insecurity; low block coverage - check sub-parts are complete; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
+          <t>explain insecurity; low block coverage - check sub-parts are complete; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling; topic inherited from sibling</t>
         </is>
       </c>
       <c r="K879" t="inlineStr">
@@ -49692,11 +49692,14 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="8">
+  <dataValidations count="9">
     <dataValidation sqref="E2:E862" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Objective (MCQ),Short answer,Explanation/Theory,Calculation,Diagram/Label,Case study,Comparison/Discussion,Other"</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E862" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"compute,draw/diagram,compare,list/enumerate,scenario/justify,short objective,define/explain"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E2:E892" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"compute,draw/diagram,compare,list/enumerate,scenario/justify,short objective,define/explain"</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E892" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">

</xml_diff>